<commit_message>
changed project directory structure
</commit_message>
<xml_diff>
--- a/templates/template_upload_excel.xlsx
+++ b/templates/template_upload_excel.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LPiGK\Desktop\Flavia Leotta\lab_database\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LPiGK\Desktop\Flavia Leotta\lab_database\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{563BA108-10EB-4628-B0D7-EC6E9939D25B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93C49342-DB28-483A-B081-BA2FE71E8765}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{CFC8A868-97A3-4117-AEBD-5D527B3D440E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="9" xr2:uid="{CFC8A868-97A3-4117-AEBD-5D527B3D440E}"/>
   </bookViews>
   <sheets>
     <sheet name="sampling_sites" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="80">
   <si>
     <t>site_name</t>
   </si>
@@ -284,6 +284,9 @@
   </si>
   <si>
     <t>qpcr_remarks</t>
+  </si>
+  <si>
+    <t>unique_reads_map</t>
   </si>
 </sst>
 </file>
@@ -665,17 +668,17 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5454034-6535-4BFE-BCAB-60921B85BD73}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.42578125" style="1" customWidth="1"/>
     <col min="2" max="2" width="11.140625" style="1" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="16.5703125" customWidth="1"/>
-    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="4" max="5" width="16.5703125" customWidth="1"/>
+    <col min="6" max="6" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>48</v>
       </c>
@@ -689,6 +692,9 @@
         <v>61</v>
       </c>
       <c r="E1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F1" t="s">
         <v>62</v>
       </c>
     </row>

</xml_diff>